<commit_message>
Update CBase Description method and Related Class.
</commit_message>
<xml_diff>
--- a/Experts/Anhnt/Document/MQL5 Note/2026 0407 MVC Refactor.xlsx
+++ b/Experts/Anhnt/Document/MQL5 Note/2026 0407 MVC Refactor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\AppData\Roaming\MetaQuotes\Terminal\D0E8209F77C8CF37AD8BF550E51FF075\MQL5\Experts\Anhnt\Document\MQL5 Note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898017B0-7FED-414F-9C6A-64D397C4AC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74FB35D7-2201-4EE6-A6DC-253F8E7DA643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{5B521979-E0DC-4D73-A935-0CEFCD7B0287}"/>
   </bookViews>
@@ -441,7 +441,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -463,6 +463,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -494,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -503,16 +509,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -530,6 +530,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2238,1010 +2250,1010 @@
     <col min="1" max="1" width="15.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.33203125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="10" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.33203125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="6" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="11" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="6"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="7" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="7"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="7" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F4" s="7"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="9" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="F6" s="7"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="11" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F8" s="7"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F9" s="7"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="7"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F11" s="7"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="7"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="7"/>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F14" s="7"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="F15" s="7"/>
+      <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F16" s="7"/>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="7" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="7"/>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="7" t="s">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F18" s="7"/>
+      <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="7" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="7"/>
+      <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F20" s="7"/>
+      <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F21" s="7"/>
+      <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="7"/>
+      <c r="F22" s="5"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F23" s="7"/>
+      <c r="F23" s="5"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="7"/>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="7"/>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="7"/>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F27" s="7"/>
+      <c r="F27" s="5"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="7" t="s">
+      <c r="A28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F28" s="7"/>
+      <c r="F28" s="5"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="7" t="s">
+      <c r="A29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F29" s="7"/>
+      <c r="F29" s="5"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" s="10" t="s">
+      <c r="A30" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F30" s="9"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="5" t="s">
+      <c r="A31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="F31" s="7"/>
+      <c r="F31" s="5"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="5" t="s">
+      <c r="A32" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E32" s="7" t="s">
+      <c r="D32" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F32" s="7"/>
+      <c r="F32" s="5"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B33" s="5" t="s">
+      <c r="A33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E33" s="7" t="s">
+      <c r="D33" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F33" s="7"/>
+      <c r="F33" s="5"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="5" t="s">
+      <c r="A34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E34" s="7" t="s">
+      <c r="D34" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E34" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F34" s="7"/>
+      <c r="F34" s="5"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B35" s="5" t="s">
+      <c r="A35" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E35" s="7" t="s">
+      <c r="D35" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F35" s="7"/>
+      <c r="F35" s="5"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B36" s="5" t="s">
+      <c r="A36" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E36" s="7" t="s">
+      <c r="D36" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F36" s="7"/>
+      <c r="F36" s="5"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37" s="5" t="s">
+      <c r="A37" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E37" s="7" t="s">
+      <c r="D37" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E37" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F37" s="7"/>
+      <c r="F37" s="5"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B38" s="5" t="s">
+      <c r="A38" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D38" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E38" s="7" t="s">
+      <c r="D38" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E38" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F38" s="7"/>
+      <c r="F38" s="5"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B39" s="5" t="s">
+      <c r="A39" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E39" s="7" t="s">
+      <c r="D39" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E39" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="F39" s="7"/>
+      <c r="F39" s="5"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B40" s="5" t="s">
+      <c r="A40" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D40" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E40" s="7" t="s">
+      <c r="D40" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E40" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F40" s="7"/>
+      <c r="F40" s="5"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B41" s="5" t="s">
+      <c r="A41" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E41" s="7" t="s">
+      <c r="D41" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E41" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F41" s="7"/>
+      <c r="F41" s="5"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B42" s="5" t="s">
+      <c r="A42" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D42" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E42" s="7" t="s">
+      <c r="D42" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F42" s="7"/>
+      <c r="F42" s="5"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B43" s="5" t="s">
+      <c r="A43" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E43" s="7" t="s">
+      <c r="D43" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F43" s="7"/>
+      <c r="F43" s="5"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B44" s="5" t="s">
+      <c r="A44" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D44" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E44" s="7" t="s">
+      <c r="D44" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E44" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F44" s="7"/>
+      <c r="F44" s="5"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" s="5" t="s">
+      <c r="A45" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E45" s="7" t="s">
+      <c r="D45" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F45" s="7"/>
+      <c r="F45" s="5"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B46" s="5" t="s">
+      <c r="A46" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E46" s="7" t="s">
+      <c r="D46" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F46" s="7"/>
+      <c r="F46" s="5"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B47" s="5" t="s">
+      <c r="A47" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D47" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E47" s="7" t="s">
+      <c r="D47" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F47" s="7"/>
+      <c r="F47" s="5"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B48" s="5" t="s">
+      <c r="A48" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D48" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E48" s="7" t="s">
+      <c r="D48" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E48" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F48" s="7"/>
+      <c r="F48" s="5"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B49" s="5" t="s">
+      <c r="A49" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C49" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D49" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E49" s="7" t="s">
+      <c r="D49" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E49" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F49" s="7"/>
+      <c r="F49" s="5"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B50" s="5" t="s">
+      <c r="A50" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D50" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E50" s="7" t="s">
+      <c r="D50" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E50" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F50" s="7"/>
+      <c r="F50" s="5"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B51" s="5" t="s">
+      <c r="A51" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D51" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E51" s="7" t="s">
+      <c r="D51" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F51" s="7"/>
+      <c r="F51" s="5"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B52" s="5" t="s">
+      <c r="A52" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D52" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E52" s="7" t="s">
+      <c r="D52" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E52" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F52" s="7"/>
+      <c r="F52" s="5"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B53" s="5" t="s">
+      <c r="A53" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D53" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E53" s="7" t="s">
+      <c r="D53" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E53" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F53" s="7"/>
+      <c r="F53" s="5"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B54" s="5" t="s">
+      <c r="A54" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D54" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E54" s="7" t="s">
+      <c r="D54" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E54" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F54" s="7"/>
+      <c r="F54" s="5"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B55" s="5" t="s">
+      <c r="A55" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D55" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="7" t="s">
+      <c r="D55" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E55" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F55" s="7"/>
+      <c r="F55" s="5"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B56" s="5" t="s">
+      <c r="A56" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D56" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E56" s="7" t="s">
+      <c r="D56" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F56" s="7"/>
+      <c r="F56" s="5"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B57" s="5" t="s">
+      <c r="A57" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B57" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C57" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D57" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E57" s="7" t="s">
+      <c r="D57" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E57" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="F57" s="7"/>
+      <c r="F57" s="5"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B58" s="5" t="s">
+      <c r="A58" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B58" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E58" s="7" t="s">
+      <c r="D58" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E58" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F58" s="7"/>
+      <c r="F58" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>